<commit_message>
hoàn chỉnh phân công, thêm mới các thư mục
</commit_message>
<xml_diff>
--- a/WBS/WBS_G9.xlsx
+++ b/WBS/WBS_G9.xlsx
@@ -4,10 +4,10 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="16836" windowHeight="9144"/>
+    <workbookView windowWidth="12276" windowHeight="8556"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="NhiemVu" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,6 +26,128 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+  <si>
+    <t>Ngày bắt đầu</t>
+  </si>
+  <si>
+    <t>Ngày kết thúc</t>
+  </si>
+  <si>
+    <t>27/10/2006</t>
+  </si>
+  <si>
+    <t>Nội dung</t>
+  </si>
+  <si>
+    <t>Bắt đầu</t>
+  </si>
+  <si>
+    <t>Kết thúc</t>
+  </si>
+  <si>
+    <t>Phụ trách</t>
+  </si>
+  <si>
+    <t>Trạng thái</t>
+  </si>
+  <si>
+    <t>Mô tả</t>
+  </si>
+  <si>
+    <t>Phân công nhiệm vụ, theo dõi kiểm tra nội dung, sửa, viết báo cáo tổng hợp nội dung cuối cùng</t>
+  </si>
+  <si>
+    <t>Nguyễn Chánh Tư Duy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. MỞ ĐẦU
+- Lý do chọn đề tài(dẫn dắt vào nơi cụ thể cần khảo sát
+- Vấn đề nghiêm trọng về ùn tắt giao thông tại Việt Nam
+2. CHƯƠNG 1: TỔNG QUAN ĐỀ TÀI
+1.1. Mục tiêu của đề tài(khảo sát thực trạng,  )
+1.2. Phạm vi nghiên cứu(vị trí, thời gian, số liệu ) có hình ảnh
+</t>
+  </si>
+  <si>
+    <t>Lê Doãn Đạt</t>
+  </si>
+  <si>
+    <t>Phải xác định
+sớm vị trí thực tế khảo sát, chậm nhất sau 2 ngày nhận nhiệm vụ</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">3. CHƯƠNG 2: CƠ SỞ LÝ THUYẾT
+2.1. Tổng quan về ITS
+(ITS là gì? Thành phần của ITS, Vai trò của ITS trong giao thông.)
+2.2. Các khái niệm về ùn tắc
+2.3. Các yếu tố gây ùn tắc
+2.4. Các phương pháp </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="163"/>
+      </rPr>
+      <t>đánh giá</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="163"/>
+      </rPr>
+      <t xml:space="preserve"> ùn tắc (Lưu lượng xe, thời gian chờ, độ dài hàng xe, vận tốc, hình ảnh/video...)</t>
+    </r>
+  </si>
+  <si>
+    <t>Nguyễn Minh Hiếu</t>
+  </si>
+  <si>
+    <t>4. CHƯƠNG 3: PHÂN TÍCH VÀ TRIỂN KHAI
+3.1. Mô tả khu vực khảo sát
+3.2. Thu thập dữ liệu thực tế (Lưu lượng xe, thời gian chờ, độ dài hàng xe, vận tốc, hình ảnh/video.)
+3.3. Problem modelling (vẽ sơ đồ cơ bản vấn đề)
+3.4. Phân tích nguyên nhân</t>
+  </si>
+  <si>
+    <t>Lê Tấn Đạt</t>
+  </si>
+  <si>
+    <t>5. CHƯƠNG 4: ĐÁNH GIÁ VÀ ĐỀ XUẤT
+4.1. Điểm mạnh, hạn chế (của kết quả khảo sát thực tế)
+4.2. Yêu cầu hạ tầng, chi phí và điều kiện áp dụng
+4.3. Rào cản
+4.4. 5 tiêu chí kỹ sư ITS
+4.5. Giải pháp/đề xuất của nhóm
+6. Chương 5: KẾT LUẬN 
+Tóm lại hu vực khảo sát có tình trạng ùn tắc như thế nào?
+5.1. Ý nghĩa đối với ngành ITS
+5.2. Kết luận chung</t>
+  </si>
+  <si>
+    <t>Nguyễn Xuân Thủy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
@@ -34,10 +156,24 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -186,8 +322,15 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="163"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -196,6 +339,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor theme="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor theme="5" tint="0.799981688894314"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor theme="4" tint="0.599993896298105"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor theme="4" tint="0.799981688894314"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -381,11 +554,178 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="22">
     <border>
       <left/>
       <right/>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thick">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thick">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -507,139 +847,214 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="58" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -921,15 +1336,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>53340</xdr:colOff>
+      <xdr:colOff>1877060</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:rowOff>163830</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>579120</xdr:colOff>
+      <xdr:colOff>45085</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -938,12 +1353,18 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="381000" y="114300"/>
-          <a:ext cx="2354580" cy="365760"/>
+          <a:off x="2204720" y="163830"/>
+          <a:ext cx="2854325" cy="363855"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
         </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent3">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="2">
@@ -963,16 +1384,23 @@
       </xdr:style>
       <xdr:txBody>
         <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
-            <a:rPr lang="en-US" sz="1600">
+            <a:rPr lang="en-US" sz="2000">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
               <a:latin typeface="Times New Roman" panose="02020603050405020304" charset="0"/>
               <a:cs typeface="Times New Roman" panose="02020603050405020304" charset="0"/>
             </a:rPr>
             <a:t>Quản lý tiểu luận nhóm 9</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1600">
+          <a:endParaRPr lang="en-US" sz="2000">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
             <a:latin typeface="Times New Roman" panose="02020603050405020304" charset="0"/>
             <a:cs typeface="Times New Roman" panose="02020603050405020304" charset="0"/>
           </a:endParaRPr>
@@ -1234,12 +1662,205 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.77777777777778" customWidth="1"/>
+    <col min="2" max="2" width="51.8888888888889" customWidth="1"/>
+    <col min="3" max="3" width="7.88888888888889" customWidth="1"/>
+    <col min="4" max="4" width="8.55555555555556" customWidth="1"/>
+    <col min="5" max="5" width="20.2222222222222" customWidth="1"/>
+    <col min="6" max="6" width="11.7777777777778" customWidth="1"/>
+    <col min="7" max="7" width="13.2222222222222" customWidth="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="3">
+        <v>46336</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" ht="15.15" spans="1:12">
+      <c r="A5" s="1"/>
+      <c r="B5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" ht="40.8" customHeight="1" spans="1:12">
+      <c r="A6" s="1"/>
+      <c r="B6" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="9">
+        <v>46306</v>
+      </c>
+      <c r="D6" s="9">
+        <v>46321</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="10"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+    </row>
+    <row r="7" ht="100.8" spans="1:12">
+      <c r="A7" s="1"/>
+      <c r="B7" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="13">
+        <v>46306</v>
+      </c>
+      <c r="D7" s="13">
+        <v>46313</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="14"/>
+      <c r="G7" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+    </row>
+    <row r="8" ht="127" customHeight="1" spans="1:12">
+      <c r="A8" s="1"/>
+      <c r="B8" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="17">
+        <v>46306</v>
+      </c>
+      <c r="D8" s="17">
+        <v>46315</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="18"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="L8" s="20"/>
+    </row>
+    <row r="9" ht="92" customHeight="1" spans="1:12">
+      <c r="A9" s="1"/>
+      <c r="B9" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="13">
+        <v>46306</v>
+      </c>
+      <c r="D9" s="13">
+        <v>46319</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="14"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+    </row>
+    <row r="10" ht="150" customHeight="1" spans="1:12">
+      <c r="A10" s="1"/>
+      <c r="B10" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="22">
+        <v>46306</v>
+      </c>
+      <c r="D10" s="22">
+        <v>46320</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="23"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+    </row>
+    <row r="11" ht="17" customHeight="1" spans="1:12">
+      <c r="A11" s="1"/>
+      <c r="B11" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Kiểm tra hoàn thành phần Mở đầu & Chương1
</commit_message>
<xml_diff>
--- a/WBS/WBS_G9.xlsx
+++ b/WBS/WBS_G9.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="12276" windowHeight="8556"/>
+    <workbookView windowWidth="22188" windowHeight="9084"/>
   </bookViews>
   <sheets>
     <sheet name="NhiemVu" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Ngày bắt đầu</t>
   </si>
@@ -72,6 +72,9 @@
   </si>
   <si>
     <t>Lê Doãn Đạt</t>
+  </si>
+  <si>
+    <t>Đã hoàn thành</t>
   </si>
   <si>
     <t>Phải xác định
@@ -156,7 +159,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -174,6 +177,13 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -847,137 +857,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1023,6 +1033,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1035,6 +1048,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -1048,6 +1064,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
@@ -1670,7 +1689,7 @@
     <col min="3" max="3" width="7.88888888888889" customWidth="1"/>
     <col min="4" max="4" width="8.55555555555556" customWidth="1"/>
     <col min="5" max="5" width="20.2222222222222" customWidth="1"/>
-    <col min="6" max="6" width="11.7777777777778" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="13.2222222222222" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1777,80 +1796,82 @@
         <v>46306</v>
       </c>
       <c r="D7" s="13">
-        <v>46313</v>
+        <v>46315</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="15" t="s">
+      <c r="F7" s="15" t="s">
         <v>13</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>14</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
     </row>
     <row r="8" ht="127" customHeight="1" spans="1:12">
       <c r="A8" s="1"/>
-      <c r="B8" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="17">
+      <c r="B8" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="18">
         <v>46306</v>
       </c>
-      <c r="D8" s="17">
-        <v>46315</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="18"/>
-      <c r="G8" s="19"/>
+      <c r="D8" s="18">
+        <v>46321</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
-      <c r="L8" s="20"/>
+      <c r="L8" s="22"/>
     </row>
     <row r="9" ht="92" customHeight="1" spans="1:12">
       <c r="A9" s="1"/>
       <c r="B9" s="12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" s="13">
         <v>46306</v>
       </c>
       <c r="D9" s="13">
-        <v>46319</v>
+        <v>46321</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="15"/>
+        <v>18</v>
+      </c>
+      <c r="F9" s="15"/>
+      <c r="G9" s="16"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
     </row>
     <row r="10" ht="150" customHeight="1" spans="1:12">
       <c r="A10" s="1"/>
-      <c r="B10" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" s="22">
+      <c r="B10" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="24">
         <v>46306</v>
       </c>
-      <c r="D10" s="22">
-        <v>46320</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="24"/>
+      <c r="D10" s="24">
+        <v>46321</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="26"/>
+      <c r="G10" s="27"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
     </row>
     <row r="11" ht="17" customHeight="1" spans="1:12">
       <c r="A11" s="1"/>
-      <c r="B11" s="25" t="s">
-        <v>20</v>
+      <c r="B11" s="28" t="s">
+        <v>21</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>

</xml_diff>